<commit_message>
feat: Se agrego un modelo de IA optimizado para tener un mejor manejo de los umbrales para la prediccion de desercion de los estudiantes
</commit_message>
<xml_diff>
--- a/AI/Proyecto_Desercion_Escolar/comparacion/comparacion_metricas.xlsx
+++ b/AI/Proyecto_Desercion_Escolar/comparacion/comparacion_metricas.xlsx
@@ -617,10 +617,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>28.50906133651733</v>
+        <v>26.63079977035522</v>
       </c>
       <c r="C16" t="n">
-        <v>27.70980358123779</v>
+        <v>27.50123500823975</v>
       </c>
     </row>
   </sheetData>

</xml_diff>